<commit_message>
Mudei o navegador para CHROME
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sotreqcloud-my.sharepoint.com/personal/darlan_s_monteiro_sotreq_com_br/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\700543\Sotreq\Darlan Monteiro - Desenvolvimento\status_project\STATUS-DE-COMUNICACAO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{31F0481F-6BEE-474B-8442-46A54322DFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59DCED67-45ED-5EC0-BDD4-8CE099AC3C31}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5BCE632-FE67-4EB9-92B2-4F3365AFE9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,126 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
-  <si>
-    <t>Barra Do Para</t>
-  </si>
-  <si>
-    <t>Belov</t>
-  </si>
-  <si>
-    <t>Brasbunker</t>
-  </si>
-  <si>
-    <t>Cargill</t>
-  </si>
-  <si>
-    <t>CBO</t>
-  </si>
-  <si>
-    <t>Chibatao</t>
-  </si>
-  <si>
-    <t>Cidade Transporte</t>
-  </si>
-  <si>
-    <t>Comando Da Marinha</t>
-  </si>
-  <si>
-    <t>Fugro</t>
-  </si>
-  <si>
-    <t>Halliburton Brasil</t>
-  </si>
-  <si>
-    <t>Hermasa</t>
-  </si>
-  <si>
-    <t>Hidrovias Do Brasil</t>
-  </si>
-  <si>
-    <t>Internav Navegacao LTDA</t>
-  </si>
-  <si>
-    <t>Majonav</t>
-  </si>
-  <si>
-    <t>MORRIS DAYAN</t>
-  </si>
-  <si>
-    <t>MRS Logistica S/A</t>
-  </si>
-  <si>
-    <t>Muliceiro</t>
-  </si>
-  <si>
-    <t>NAVEGACOES UNIDAS TAPAJOS</t>
-  </si>
-  <si>
-    <t>Nortelog</t>
-  </si>
-  <si>
-    <t>Oceanpact</t>
-  </si>
-  <si>
-    <t>Ocidental Transportes</t>
-  </si>
-  <si>
-    <t>PERBRAS EMP BRAS DE PERFURAC</t>
-  </si>
-  <si>
-    <t>Petro Rio</t>
-  </si>
-  <si>
-    <t>Petrobras</t>
-  </si>
-  <si>
-    <t>PetroReconcavo</t>
-  </si>
-  <si>
-    <t>Ragnar</t>
-  </si>
-  <si>
-    <t>Rumo Logistica</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>SAAM Towage</t>
-  </si>
-  <si>
-    <t>SC Transportes E Construcoesltda</t>
-  </si>
-  <si>
-    <t>SIEM OFFSHORE DO BRASIL</t>
-  </si>
-  <si>
-    <t>Silnave Navegacao</t>
-  </si>
-  <si>
-    <t>Svitzer AMS</t>
-  </si>
-  <si>
-    <t>Transportadora Brasileira Gasoduto</t>
-  </si>
-  <si>
-    <t>Vale S/A</t>
-  </si>
-  <si>
-    <t>Waldemiro Lustosa</t>
   </si>
   <si>
     <t>Wilson Sons</t>
   </si>
   <si>
     <t>Clientes</t>
-  </si>
-  <si>
-    <t>Hygge</t>
-  </si>
-  <si>
-    <t>LOUIS DREYFUS COMPANY</t>
-  </si>
-  <si>
-    <t>Tidewater</t>
   </si>
 </sst>
 </file>
@@ -228,10 +117,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F814540-4107-4737-8705-94C4B19FE763}" name="Clientes" displayName="Clientes" ref="A1:A40" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:A40" xr:uid="{7F814540-4107-4737-8705-94C4B19FE763}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A40">
-    <sortCondition ref="A1:A40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7F814540-4107-4737-8705-94C4B19FE763}" name="Clientes" displayName="Clientes" ref="A1:A3" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:A3" xr:uid="{7F814540-4107-4737-8705-94C4B19FE763}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A3">
+    <sortCondition ref="A1:A3"/>
   </sortState>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{EB5712E7-D126-48A0-9D53-B4B87ED0A711}" name="Clientes"/>
@@ -503,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.1796875" bestFit="1" customWidth="1"/>
@@ -511,7 +400,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
@@ -524,191 +413,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>35</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -718,26 +422,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3507f5ad-155e-4a06-8dc0-2b64038b46b7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b06b84b9-f542-449b-8b93-9e89166b9480" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010045BA7E4D780EAE42A37D6F8C1A49608E" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="4cc85f28385ad9aa4feaf1e5a101789d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3507f5ad-155e-4a06-8dc0-2b64038b46b7" xmlns:ns3="b06b84b9-f542-449b-8b93-9e89166b9480" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e1ecea972f00b60911b6311a5ade6ca1" ns2:_="" ns3:_="">
     <xsd:import namespace="3507f5ad-155e-4a06-8dc0-2b64038b46b7"/>
@@ -972,26 +656,27 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3507f5ad-155e-4a06-8dc0-2b64038b46b7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b06b84b9-f542-449b-8b93-9e89166b9480" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E4530B-9FBF-4C17-91D2-4949D659C036}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3507f5ad-155e-4a06-8dc0-2b64038b46b7"/>
-    <ds:schemaRef ds:uri="b06b84b9-f542-449b-8b93-9e89166b9480"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D848A61B-71DE-4A15-BFAF-84FA92AE61F6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD46B981-9627-468A-9A6C-D4ED1EC5B2B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1008,4 +693,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D848A61B-71DE-4A15-BFAF-84FA92AE61F6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64E4530B-9FBF-4C17-91D2-4949D659C036}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3507f5ad-155e-4a06-8dc0-2b64038b46b7"/>
+    <ds:schemaRef ds:uri="b06b84b9-f542-449b-8b93-9e89166b9480"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>